<commit_message>
feat(examples): reference port of the settlement macro, its API and a shadcn-svelte form
The Python port reproduces the macro day by day (characterization tests against expected/settlement.csv) and reports the hour without price the macro settled at 0 silently. The FastAPI request model is the only definition of the inputs: the SvelteKit form reads it from openapi.json, Superforms validates with it in the browser and on the server (schemasafe), shadcn-svelte draws the controls, and broken rules become sentences with the limits taken from the schema.
</commit_message>
<xml_diff>
--- a/examples/settlement/settlement.xlsx
+++ b/examples/settlement/settlement.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sota/repos/datons/excel/examples/settlement/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_F986D1BD58B48FE16C6B1B6285CC0AE1D725702B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Parametros" sheetId="1" r:id="rId1"/>
@@ -18,20 +12,7 @@
     <sheet name="Precios" sheetId="3" r:id="rId3"/>
     <sheet name="Liquidacion" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -92,12 +73,12 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -145,21 +126,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -197,7 +170,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -231,7 +204,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -266,10 +238,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -442,15 +413,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="18.6640625" customWidth="1"/>
-    <col min="3" max="3" width="44.6640625" customWidth="1"/>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="3" max="3" width="44.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -461,18 +432,18 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="2">
-        <v>4.4999999999999998E-2</v>
+        <v>0.045</v>
       </c>
       <c r="C2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -483,7 +454,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -498,15 +469,15 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D98"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12.6640625" customWidth="1"/>
-    <col min="2" max="4" width="14.6640625" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="4" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
@@ -520,7 +491,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4">
       <c r="A2" s="3">
         <v>46319</v>
       </c>
@@ -531,11 +502,11 @@
         <v>4.2</v>
       </c>
       <c r="D2">
-        <f t="shared" ref="D2:D33" si="0">C2/1000</f>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C2/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" s="3">
         <v>46319</v>
       </c>
@@ -546,11 +517,11 @@
         <v>4.2</v>
       </c>
       <c r="D3">
-        <f t="shared" si="0"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C3/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
       <c r="A4" s="3">
         <v>46319</v>
       </c>
@@ -561,11 +532,11 @@
         <v>4.2</v>
       </c>
       <c r="D4">
-        <f t="shared" si="0"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C4/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
       <c r="A5" s="3">
         <v>46319</v>
       </c>
@@ -576,11 +547,11 @@
         <v>4.2</v>
       </c>
       <c r="D5">
-        <f t="shared" si="0"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C5/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
       <c r="A6" s="3">
         <v>46319</v>
       </c>
@@ -591,11 +562,11 @@
         <v>4.2</v>
       </c>
       <c r="D6">
-        <f t="shared" si="0"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C6/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
       <c r="A7" s="3">
         <v>46319</v>
       </c>
@@ -606,11 +577,11 @@
         <v>4.2</v>
       </c>
       <c r="D7">
-        <f t="shared" si="0"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C7/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
       <c r="A8" s="3">
         <v>46319</v>
       </c>
@@ -621,11 +592,11 @@
         <v>4.2</v>
       </c>
       <c r="D8">
-        <f t="shared" si="0"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C8/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
       <c r="A9" s="3">
         <v>46319</v>
       </c>
@@ -636,11 +607,11 @@
         <v>250.596</v>
       </c>
       <c r="D9">
-        <f t="shared" si="0"/>
-        <v>0.25059599999999999</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C9/1000</f>
+        <v>0.250596</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
       <c r="A10" s="3">
         <v>46319</v>
       </c>
@@ -651,11 +622,11 @@
         <v>480.2</v>
       </c>
       <c r="D10">
-        <f t="shared" si="0"/>
-        <v>0.48020000000000002</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C10/1000</f>
+        <v>0.4802</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
       <c r="A11" s="3">
         <v>46319</v>
       </c>
@@ -663,14 +634,14 @@
         <v>10</v>
       </c>
       <c r="C11">
-        <v>677.36599999999999</v>
+        <v>677.366</v>
       </c>
       <c r="D11">
-        <f t="shared" si="0"/>
-        <v>0.67736600000000002</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C11/1000</f>
+        <v>0.677366</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
       <c r="A12" s="3">
         <v>46319</v>
       </c>
@@ -678,14 +649,14 @@
         <v>11</v>
       </c>
       <c r="C12">
-        <v>828.65599999999995</v>
+        <v>828.6559999999999</v>
       </c>
       <c r="D12">
-        <f t="shared" si="0"/>
-        <v>0.82865599999999995</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C12/1000</f>
+        <v>0.828656</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
       <c r="A13" s="3">
         <v>46319</v>
       </c>
@@ -693,14 +664,14 @@
         <v>12</v>
       </c>
       <c r="C13">
-        <v>923.76099999999997</v>
+        <v>923.761</v>
       </c>
       <c r="D13">
-        <f t="shared" si="0"/>
-        <v>0.92376099999999994</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C13/1000</f>
+        <v>0.9237609999999999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
       <c r="A14" s="3">
         <v>46319</v>
       </c>
@@ -711,11 +682,11 @@
         <v>956.2</v>
       </c>
       <c r="D14">
-        <f t="shared" si="0"/>
-        <v>0.95620000000000005</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C14/1000</f>
+        <v>0.9562</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
       <c r="A15" s="3">
         <v>46319</v>
       </c>
@@ -723,14 +694,14 @@
         <v>14</v>
       </c>
       <c r="C15">
-        <v>923.76099999999997</v>
+        <v>923.761</v>
       </c>
       <c r="D15">
-        <f t="shared" si="0"/>
-        <v>0.92376099999999994</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C15/1000</f>
+        <v>0.9237609999999999</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
       <c r="A16" s="3">
         <v>46319</v>
       </c>
@@ -738,14 +709,14 @@
         <v>15</v>
       </c>
       <c r="C16">
-        <v>828.65599999999995</v>
+        <v>828.6559999999999</v>
       </c>
       <c r="D16">
-        <f t="shared" si="0"/>
-        <v>0.82865599999999995</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C16/1000</f>
+        <v>0.828656</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
       <c r="A17" s="3">
         <v>46319</v>
       </c>
@@ -753,14 +724,14 @@
         <v>16</v>
       </c>
       <c r="C17">
-        <v>677.36599999999999</v>
+        <v>677.366</v>
       </c>
       <c r="D17">
-        <f t="shared" si="0"/>
-        <v>0.67736600000000002</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C17/1000</f>
+        <v>0.677366</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
       <c r="A18" s="3">
         <v>46319</v>
       </c>
@@ -771,11 +742,11 @@
         <v>480.2</v>
       </c>
       <c r="D18">
-        <f t="shared" si="0"/>
-        <v>0.48020000000000002</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C18/1000</f>
+        <v>0.4802</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
       <c r="A19" s="3">
         <v>46319</v>
       </c>
@@ -786,11 +757,11 @@
         <v>250.596</v>
       </c>
       <c r="D19">
-        <f t="shared" si="0"/>
-        <v>0.25059599999999999</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C19/1000</f>
+        <v>0.250596</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
       <c r="A20" s="3">
         <v>46319</v>
       </c>
@@ -801,11 +772,11 @@
         <v>4.2</v>
       </c>
       <c r="D20">
-        <f t="shared" si="0"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C20/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
       <c r="A21" s="3">
         <v>46319</v>
       </c>
@@ -816,11 +787,11 @@
         <v>4.2</v>
       </c>
       <c r="D21">
-        <f t="shared" si="0"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C21/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
       <c r="A22" s="3">
         <v>46319</v>
       </c>
@@ -831,11 +802,11 @@
         <v>4.2</v>
       </c>
       <c r="D22">
-        <f t="shared" si="0"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C22/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
       <c r="A23" s="3">
         <v>46319</v>
       </c>
@@ -846,11 +817,11 @@
         <v>4.2</v>
       </c>
       <c r="D23">
-        <f t="shared" si="0"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C23/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
       <c r="A24" s="3">
         <v>46319</v>
       </c>
@@ -861,11 +832,11 @@
         <v>4.2</v>
       </c>
       <c r="D24">
-        <f t="shared" si="0"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C24/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
       <c r="A25" s="3">
         <v>46319</v>
       </c>
@@ -876,11 +847,11 @@
         <v>4.2</v>
       </c>
       <c r="D25">
-        <f t="shared" si="0"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C25/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
       <c r="A26" s="3">
         <v>46320</v>
       </c>
@@ -891,11 +862,11 @@
         <v>4.2</v>
       </c>
       <c r="D26">
-        <f t="shared" si="0"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C26/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
       <c r="A27" s="3">
         <v>46320</v>
       </c>
@@ -906,11 +877,11 @@
         <v>4.2</v>
       </c>
       <c r="D27">
-        <f t="shared" si="0"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C27/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
       <c r="A28" s="3">
         <v>46320</v>
       </c>
@@ -921,11 +892,11 @@
         <v>4.2</v>
       </c>
       <c r="D28">
-        <f t="shared" si="0"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C28/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
       <c r="A29" s="3">
         <v>46320</v>
       </c>
@@ -936,11 +907,11 @@
         <v>4.2</v>
       </c>
       <c r="D29">
-        <f t="shared" si="0"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C29/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
       <c r="A30" s="3">
         <v>46320</v>
       </c>
@@ -951,11 +922,11 @@
         <v>4.2</v>
       </c>
       <c r="D30">
-        <f t="shared" si="0"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C30/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
       <c r="A31" s="3">
         <v>46320</v>
       </c>
@@ -966,11 +937,11 @@
         <v>4.2</v>
       </c>
       <c r="D31">
-        <f t="shared" si="0"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C31/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4">
       <c r="A32" s="3">
         <v>46320</v>
       </c>
@@ -981,11 +952,11 @@
         <v>4.2</v>
       </c>
       <c r="D32">
-        <f t="shared" si="0"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C32/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
       <c r="A33" s="3">
         <v>46320</v>
       </c>
@@ -996,11 +967,11 @@
         <v>224.196</v>
       </c>
       <c r="D33">
-        <f t="shared" si="0"/>
-        <v>0.22419600000000001</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C33/1000</f>
+        <v>0.224196</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4">
       <c r="A34" s="3">
         <v>46320</v>
       </c>
@@ -1011,11 +982,11 @@
         <v>429.2</v>
       </c>
       <c r="D34">
-        <f t="shared" ref="D34:D65" si="1">C34/1000</f>
+        <f>C34/1000</f>
         <v>0.42919999999999997</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:4">
       <c r="A35" s="3">
         <v>46320</v>
       </c>
@@ -1023,14 +994,14 @@
         <v>10</v>
       </c>
       <c r="C35">
-        <v>605.24099999999999</v>
+        <v>605.241</v>
       </c>
       <c r="D35">
-        <f t="shared" si="1"/>
-        <v>0.60524100000000003</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C35/1000</f>
+        <v>0.605241</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4">
       <c r="A36" s="3">
         <v>46320</v>
       </c>
@@ -1041,11 +1012,11 @@
         <v>740.322</v>
       </c>
       <c r="D36">
-        <f t="shared" si="1"/>
-        <v>0.74032200000000004</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C36/1000</f>
+        <v>0.740322</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4">
       <c r="A37" s="3">
         <v>46320</v>
       </c>
@@ -1053,14 +1024,14 @@
         <v>12</v>
       </c>
       <c r="C37">
-        <v>825.23699999999997</v>
+        <v>825.237</v>
       </c>
       <c r="D37">
-        <f t="shared" si="1"/>
+        <f>C37/1000</f>
         <v>0.825237</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:4">
       <c r="A38" s="3">
         <v>46320</v>
       </c>
@@ -1071,11 +1042,11 @@
         <v>854.2</v>
       </c>
       <c r="D38">
-        <f t="shared" si="1"/>
-        <v>0.85420000000000007</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C38/1000</f>
+        <v>0.8542000000000001</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
       <c r="A39" s="3">
         <v>46320</v>
       </c>
@@ -1083,14 +1054,14 @@
         <v>14</v>
       </c>
       <c r="C39">
-        <v>825.23699999999997</v>
+        <v>825.237</v>
       </c>
       <c r="D39">
-        <f t="shared" si="1"/>
+        <f>C39/1000</f>
         <v>0.825237</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:4">
       <c r="A40" s="3">
         <v>46320</v>
       </c>
@@ -1101,11 +1072,11 @@
         <v>740.322</v>
       </c>
       <c r="D40">
-        <f t="shared" si="1"/>
-        <v>0.74032200000000004</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C40/1000</f>
+        <v>0.740322</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4">
       <c r="A41" s="3">
         <v>46320</v>
       </c>
@@ -1113,14 +1084,14 @@
         <v>16</v>
       </c>
       <c r="C41">
-        <v>605.24099999999999</v>
+        <v>605.241</v>
       </c>
       <c r="D41">
-        <f t="shared" si="1"/>
-        <v>0.60524100000000003</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C41/1000</f>
+        <v>0.605241</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4">
       <c r="A42" s="3">
         <v>46320</v>
       </c>
@@ -1131,11 +1102,11 @@
         <v>429.2</v>
       </c>
       <c r="D42">
-        <f t="shared" si="1"/>
+        <f>C42/1000</f>
         <v>0.42919999999999997</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:4">
       <c r="A43" s="3">
         <v>46320</v>
       </c>
@@ -1146,11 +1117,11 @@
         <v>224.196</v>
       </c>
       <c r="D43">
-        <f t="shared" si="1"/>
-        <v>0.22419600000000001</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C43/1000</f>
+        <v>0.224196</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4">
       <c r="A44" s="3">
         <v>46320</v>
       </c>
@@ -1161,11 +1132,11 @@
         <v>4.2</v>
       </c>
       <c r="D44">
-        <f t="shared" si="1"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C44/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4">
       <c r="A45" s="3">
         <v>46320</v>
       </c>
@@ -1176,11 +1147,11 @@
         <v>4.2</v>
       </c>
       <c r="D45">
-        <f t="shared" si="1"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C45/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4">
       <c r="A46" s="3">
         <v>46320</v>
       </c>
@@ -1191,11 +1162,11 @@
         <v>4.2</v>
       </c>
       <c r="D46">
-        <f t="shared" si="1"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C46/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4">
       <c r="A47" s="3">
         <v>46320</v>
       </c>
@@ -1206,11 +1177,11 @@
         <v>4.2</v>
       </c>
       <c r="D47">
-        <f t="shared" si="1"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C47/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4">
       <c r="A48" s="3">
         <v>46320</v>
       </c>
@@ -1221,11 +1192,11 @@
         <v>4.2</v>
       </c>
       <c r="D48">
-        <f t="shared" si="1"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C48/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4">
       <c r="A49" s="3">
         <v>46320</v>
       </c>
@@ -1236,11 +1207,11 @@
         <v>4.2</v>
       </c>
       <c r="D49">
-        <f t="shared" si="1"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C49/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4">
       <c r="A50" s="3">
         <v>46320</v>
       </c>
@@ -1251,11 +1222,11 @@
         <v>4.2</v>
       </c>
       <c r="D50">
-        <f t="shared" si="1"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C50/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4">
       <c r="A51" s="3">
         <v>46321</v>
       </c>
@@ -1266,11 +1237,11 @@
         <v>4.2</v>
       </c>
       <c r="D51">
-        <f t="shared" si="1"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C51/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4">
       <c r="A52" s="3">
         <v>46321</v>
       </c>
@@ -1281,11 +1252,11 @@
         <v>4.2</v>
       </c>
       <c r="D52">
-        <f t="shared" si="1"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C52/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4">
       <c r="A53" s="3">
         <v>46321</v>
       </c>
@@ -1296,11 +1267,11 @@
         <v>4.2</v>
       </c>
       <c r="D53">
-        <f t="shared" si="1"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C53/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4">
       <c r="A54" s="3">
         <v>46321</v>
       </c>
@@ -1311,11 +1282,11 @@
         <v>4.2</v>
       </c>
       <c r="D54">
-        <f t="shared" si="1"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C54/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4">
       <c r="A55" s="3">
         <v>46321</v>
       </c>
@@ -1326,11 +1297,11 @@
         <v>4.2</v>
       </c>
       <c r="D55">
-        <f t="shared" si="1"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C55/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4">
       <c r="A56" s="3">
         <v>46321</v>
       </c>
@@ -1341,11 +1312,11 @@
         <v>4.2</v>
       </c>
       <c r="D56">
-        <f t="shared" si="1"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C56/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4">
       <c r="A57" s="3">
         <v>46321</v>
       </c>
@@ -1356,11 +1327,11 @@
         <v>4.2</v>
       </c>
       <c r="D57">
-        <f t="shared" si="1"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C57/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4">
       <c r="A58" s="3">
         <v>46321</v>
       </c>
@@ -1368,14 +1339,14 @@
         <v>8</v>
       </c>
       <c r="C58">
-        <v>230.79599999999999</v>
+        <v>230.796</v>
       </c>
       <c r="D58">
-        <f t="shared" si="1"/>
+        <f>C58/1000</f>
         <v>0.230796</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:4">
       <c r="A59" s="3">
         <v>46321</v>
       </c>
@@ -1383,11 +1354,11 @@
         <v>9</v>
       </c>
       <c r="D59">
-        <f t="shared" si="1"/>
+        <f>C59/1000</f>
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:4">
       <c r="A60" s="3">
         <v>46321</v>
       </c>
@@ -1395,11 +1366,11 @@
         <v>10</v>
       </c>
       <c r="D60">
-        <f t="shared" si="1"/>
+        <f>C60/1000</f>
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:4">
       <c r="A61" s="3">
         <v>46321</v>
       </c>
@@ -1407,14 +1378,14 @@
         <v>11</v>
       </c>
       <c r="C61">
-        <v>762.40499999999997</v>
+        <v>762.405</v>
       </c>
       <c r="D61">
-        <f t="shared" si="1"/>
+        <f>C61/1000</f>
         <v>0.762405</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:4">
       <c r="A62" s="3">
         <v>46321</v>
       </c>
@@ -1422,14 +1393,14 @@
         <v>12</v>
       </c>
       <c r="C62">
-        <v>849.86800000000005</v>
+        <v>849.8680000000001</v>
       </c>
       <c r="D62">
-        <f t="shared" si="1"/>
-        <v>0.84986800000000007</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C62/1000</f>
+        <v>0.8498680000000001</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4">
       <c r="A63" s="3">
         <v>46321</v>
       </c>
@@ -1440,11 +1411,11 @@
         <v>879.7</v>
       </c>
       <c r="D63">
-        <f t="shared" si="1"/>
-        <v>0.87970000000000004</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C63/1000</f>
+        <v>0.8797</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4">
       <c r="A64" s="3">
         <v>46321</v>
       </c>
@@ -1452,14 +1423,14 @@
         <v>14</v>
       </c>
       <c r="C64">
-        <v>849.86800000000005</v>
+        <v>849.8680000000001</v>
       </c>
       <c r="D64">
-        <f t="shared" si="1"/>
-        <v>0.84986800000000007</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C64/1000</f>
+        <v>0.8498680000000001</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4">
       <c r="A65" s="3">
         <v>46321</v>
       </c>
@@ -1467,14 +1438,14 @@
         <v>15</v>
       </c>
       <c r="C65">
-        <v>762.40499999999997</v>
+        <v>762.405</v>
       </c>
       <c r="D65">
-        <f t="shared" si="1"/>
+        <f>C65/1000</f>
         <v>0.762405</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:4">
       <c r="A66" s="3">
         <v>46321</v>
       </c>
@@ -1482,14 +1453,14 @@
         <v>16</v>
       </c>
       <c r="C66">
-        <v>623.27200000000005</v>
+        <v>623.272</v>
       </c>
       <c r="D66">
-        <f t="shared" ref="D66:D97" si="2">C66/1000</f>
-        <v>0.62327200000000005</v>
-      </c>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C66/1000</f>
+        <v>0.623272</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4">
       <c r="A67" s="3">
         <v>46321</v>
       </c>
@@ -1500,11 +1471,11 @@
         <v>441.95</v>
       </c>
       <c r="D67">
-        <f t="shared" si="2"/>
-        <v>0.44195000000000001</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C67/1000</f>
+        <v>0.44195</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4">
       <c r="A68" s="3">
         <v>46321</v>
       </c>
@@ -1512,14 +1483,14 @@
         <v>18</v>
       </c>
       <c r="C68">
-        <v>230.79599999999999</v>
+        <v>230.796</v>
       </c>
       <c r="D68">
-        <f t="shared" si="2"/>
+        <f>C68/1000</f>
         <v>0.230796</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:4">
       <c r="A69" s="3">
         <v>46321</v>
       </c>
@@ -1530,11 +1501,11 @@
         <v>4.2</v>
       </c>
       <c r="D69">
-        <f t="shared" si="2"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C69/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4">
       <c r="A70" s="3">
         <v>46321</v>
       </c>
@@ -1545,11 +1516,11 @@
         <v>4.2</v>
       </c>
       <c r="D70">
-        <f t="shared" si="2"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C70/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4">
       <c r="A71" s="3">
         <v>46321</v>
       </c>
@@ -1560,11 +1531,11 @@
         <v>4.2</v>
       </c>
       <c r="D71">
-        <f t="shared" si="2"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C71/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4">
       <c r="A72" s="3">
         <v>46321</v>
       </c>
@@ -1575,11 +1546,11 @@
         <v>4.2</v>
       </c>
       <c r="D72">
-        <f t="shared" si="2"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C72/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4">
       <c r="A73" s="3">
         <v>46321</v>
       </c>
@@ -1590,11 +1561,11 @@
         <v>4.2</v>
       </c>
       <c r="D73">
-        <f t="shared" si="2"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C73/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4">
       <c r="A74" s="3">
         <v>46321</v>
       </c>
@@ -1605,11 +1576,11 @@
         <v>4.2</v>
       </c>
       <c r="D74">
-        <f t="shared" si="2"/>
-        <v>4.2000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
+        <f>C74/1000</f>
+        <v>0.004200000000000001</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4">
       <c r="A75" s="3">
         <v>46322</v>
       </c>
@@ -1617,11 +1588,11 @@
         <v>1</v>
       </c>
       <c r="D75">
-        <f t="shared" si="2"/>
+        <f>C75/1000</f>
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:4">
       <c r="A76" s="3">
         <v>46322</v>
       </c>
@@ -1629,11 +1600,11 @@
         <v>2</v>
       </c>
       <c r="D76">
-        <f t="shared" si="2"/>
+        <f>C76/1000</f>
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:4">
       <c r="A77" s="3">
         <v>46322</v>
       </c>
@@ -1641,11 +1612,11 @@
         <v>3</v>
       </c>
       <c r="D77">
-        <f t="shared" si="2"/>
+        <f>C77/1000</f>
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:4">
       <c r="A78" s="3">
         <v>46322</v>
       </c>
@@ -1653,11 +1624,11 @@
         <v>4</v>
       </c>
       <c r="D78">
-        <f t="shared" si="2"/>
+        <f>C78/1000</f>
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:4">
       <c r="A79" s="3">
         <v>46322</v>
       </c>
@@ -1665,11 +1636,11 @@
         <v>5</v>
       </c>
       <c r="D79">
-        <f t="shared" si="2"/>
+        <f>C79/1000</f>
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:4">
       <c r="A80" s="3">
         <v>46322</v>
       </c>
@@ -1677,11 +1648,11 @@
         <v>6</v>
       </c>
       <c r="D80">
-        <f t="shared" si="2"/>
+        <f>C80/1000</f>
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:4">
       <c r="A81" s="3">
         <v>46322</v>
       </c>
@@ -1689,11 +1660,11 @@
         <v>7</v>
       </c>
       <c r="D81">
-        <f t="shared" si="2"/>
+        <f>C81/1000</f>
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:4">
       <c r="A82" s="3">
         <v>46322</v>
       </c>
@@ -1701,11 +1672,11 @@
         <v>8</v>
       </c>
       <c r="D82">
-        <f t="shared" si="2"/>
+        <f>C82/1000</f>
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:4">
       <c r="A83" s="3">
         <v>46322</v>
       </c>
@@ -1713,11 +1684,11 @@
         <v>9</v>
       </c>
       <c r="D83">
-        <f t="shared" si="2"/>
+        <f>C83/1000</f>
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:4">
       <c r="A84" s="3">
         <v>46322</v>
       </c>
@@ -1725,11 +1696,11 @@
         <v>10</v>
       </c>
       <c r="D84">
-        <f t="shared" si="2"/>
+        <f>C84/1000</f>
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:4">
       <c r="A85" s="3">
         <v>46322</v>
       </c>
@@ -1737,11 +1708,11 @@
         <v>11</v>
       </c>
       <c r="D85">
-        <f t="shared" si="2"/>
+        <f>C85/1000</f>
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:4">
       <c r="A86" s="3">
         <v>46322</v>
       </c>
@@ -1749,11 +1720,11 @@
         <v>12</v>
       </c>
       <c r="D86">
-        <f t="shared" si="2"/>
+        <f>C86/1000</f>
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:4">
       <c r="A87" s="3">
         <v>46322</v>
       </c>
@@ -1761,11 +1732,11 @@
         <v>13</v>
       </c>
       <c r="D87">
-        <f t="shared" si="2"/>
+        <f>C87/1000</f>
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:4">
       <c r="A88" s="3">
         <v>46322</v>
       </c>
@@ -1773,11 +1744,11 @@
         <v>14</v>
       </c>
       <c r="D88">
-        <f t="shared" si="2"/>
+        <f>C88/1000</f>
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:4">
       <c r="A89" s="3">
         <v>46322</v>
       </c>
@@ -1785,11 +1756,11 @@
         <v>15</v>
       </c>
       <c r="D89">
-        <f t="shared" si="2"/>
+        <f>C89/1000</f>
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:4">
       <c r="A90" s="3">
         <v>46322</v>
       </c>
@@ -1797,11 +1768,11 @@
         <v>16</v>
       </c>
       <c r="D90">
-        <f t="shared" si="2"/>
+        <f>C90/1000</f>
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:4">
       <c r="A91" s="3">
         <v>46322</v>
       </c>
@@ -1809,11 +1780,11 @@
         <v>17</v>
       </c>
       <c r="D91">
-        <f t="shared" si="2"/>
+        <f>C91/1000</f>
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:4">
       <c r="A92" s="3">
         <v>46322</v>
       </c>
@@ -1821,11 +1792,11 @@
         <v>18</v>
       </c>
       <c r="D92">
-        <f t="shared" si="2"/>
+        <f>C92/1000</f>
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:4">
       <c r="A93" s="3">
         <v>46322</v>
       </c>
@@ -1833,11 +1804,11 @@
         <v>19</v>
       </c>
       <c r="D93">
-        <f t="shared" si="2"/>
+        <f>C93/1000</f>
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:4">
       <c r="A94" s="3">
         <v>46322</v>
       </c>
@@ -1845,11 +1816,11 @@
         <v>20</v>
       </c>
       <c r="D94">
-        <f t="shared" si="2"/>
+        <f>C94/1000</f>
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:4">
       <c r="A95" s="3">
         <v>46322</v>
       </c>
@@ -1857,11 +1828,11 @@
         <v>21</v>
       </c>
       <c r="D95">
-        <f t="shared" si="2"/>
+        <f>C95/1000</f>
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:4">
       <c r="A96" s="3">
         <v>46322</v>
       </c>
@@ -1869,11 +1840,11 @@
         <v>22</v>
       </c>
       <c r="D96">
-        <f t="shared" si="2"/>
+        <f>C96/1000</f>
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:4">
       <c r="A97" s="3">
         <v>46322</v>
       </c>
@@ -1881,11 +1852,11 @@
         <v>23</v>
       </c>
       <c r="D97">
-        <f t="shared" si="2"/>
+        <f>C97/1000</f>
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:4">
       <c r="A98" s="3">
         <v>46322</v>
       </c>
@@ -1893,7 +1864,7 @@
         <v>24</v>
       </c>
       <c r="D98">
-        <f t="shared" ref="D98:D129" si="3">C98/1000</f>
+        <f>C98/1000</f>
         <v>0</v>
       </c>
     </row>
@@ -1903,15 +1874,15 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C97"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12.6640625" customWidth="1"/>
-    <col min="2" max="4" width="14.6640625" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="4" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
@@ -1922,7 +1893,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3">
       <c r="A2" s="3">
         <v>46319</v>
       </c>
@@ -1933,7 +1904,7 @@
         <v>83.69</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3">
       <c r="A3" s="3">
         <v>46319</v>
       </c>
@@ -1944,7 +1915,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3">
       <c r="A4" s="3">
         <v>46319</v>
       </c>
@@ -1955,7 +1926,7 @@
         <v>72.31</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3">
       <c r="A5" s="3">
         <v>46319</v>
       </c>
@@ -1966,7 +1937,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3">
       <c r="A6" s="3">
         <v>46319</v>
       </c>
@@ -1977,7 +1948,7 @@
         <v>62.44</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3">
       <c r="A7" s="3">
         <v>46319</v>
       </c>
@@ -1988,7 +1959,7 @@
         <v>58.95</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3">
       <c r="A8" s="3">
         <v>46319</v>
       </c>
@@ -1999,7 +1970,7 @@
         <v>56.75</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3">
       <c r="A9" s="3">
         <v>46319</v>
       </c>
@@ -2010,7 +1981,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3">
       <c r="A10" s="3">
         <v>46319</v>
       </c>
@@ -2021,7 +1992,7 @@
         <v>56.75</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3">
       <c r="A11" s="3">
         <v>46319</v>
       </c>
@@ -2032,7 +2003,7 @@
         <v>58.95</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3">
       <c r="A12" s="3">
         <v>46319</v>
       </c>
@@ -2043,7 +2014,7 @@
         <v>62.44</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3">
       <c r="A13" s="3">
         <v>46319</v>
       </c>
@@ -2054,7 +2025,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3">
       <c r="A14" s="3">
         <v>46319</v>
       </c>
@@ -2065,7 +2036,7 @@
         <v>72.31</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3">
       <c r="A15" s="3">
         <v>46319</v>
       </c>
@@ -2076,7 +2047,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3">
       <c r="A16" s="3">
         <v>46319</v>
       </c>
@@ -2087,7 +2058,7 @@
         <v>83.69</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:3">
       <c r="A17" s="3">
         <v>46319</v>
       </c>
@@ -2098,7 +2069,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:3">
       <c r="A18" s="3">
         <v>46319</v>
       </c>
@@ -2109,7 +2080,7 @@
         <v>93.56</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:3">
       <c r="A19" s="3">
         <v>46319</v>
       </c>
@@ -2120,7 +2091,7 @@
         <v>97.05</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:3">
       <c r="A20" s="3">
         <v>46319</v>
       </c>
@@ -2131,7 +2102,7 @@
         <v>99.25</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:3">
       <c r="A21" s="3">
         <v>46319</v>
       </c>
@@ -2142,7 +2113,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:3">
       <c r="A22" s="3">
         <v>46319</v>
       </c>
@@ -2153,7 +2124,7 @@
         <v>99.25</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:3">
       <c r="A23" s="3">
         <v>46319</v>
       </c>
@@ -2164,7 +2135,7 @@
         <v>97.05</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:3">
       <c r="A24" s="3">
         <v>46319</v>
       </c>
@@ -2175,7 +2146,7 @@
         <v>93.56</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:3">
       <c r="A25" s="3">
         <v>46319</v>
       </c>
@@ -2186,7 +2157,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:3">
       <c r="A26" s="3">
         <v>46320</v>
       </c>
@@ -2194,10 +2165,10 @@
         <v>1</v>
       </c>
       <c r="C26">
-        <v>82.99</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+        <v>82.98999999999999</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
       <c r="A27" s="3">
         <v>46320</v>
       </c>
@@ -2208,7 +2179,7 @@
         <v>77.3</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:3">
       <c r="A28" s="3">
         <v>46320</v>
       </c>
@@ -2219,7 +2190,7 @@
         <v>71.61</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:3">
       <c r="A29" s="3">
         <v>46320</v>
       </c>
@@ -2230,7 +2201,7 @@
         <v>66.3</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:3">
       <c r="A30" s="3">
         <v>46320</v>
       </c>
@@ -2241,7 +2212,7 @@
         <v>61.74</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:3">
       <c r="A31" s="3">
         <v>46320</v>
       </c>
@@ -2252,7 +2223,7 @@
         <v>58.25</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:3">
       <c r="A32" s="3">
         <v>46320</v>
       </c>
@@ -2263,7 +2234,7 @@
         <v>56.05</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:3">
       <c r="A33" s="3">
         <v>46320</v>
       </c>
@@ -2274,7 +2245,7 @@
         <v>55.3</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:3">
       <c r="A34" s="3">
         <v>46320</v>
       </c>
@@ -2285,7 +2256,7 @@
         <v>56.05</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:3">
       <c r="A35" s="3">
         <v>46320</v>
       </c>
@@ -2296,7 +2267,7 @@
         <v>58.25</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:3">
       <c r="A36" s="3">
         <v>46320</v>
       </c>
@@ -2307,7 +2278,7 @@
         <v>61.74</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:3">
       <c r="A37" s="3">
         <v>46320</v>
       </c>
@@ -2318,7 +2289,7 @@
         <v>66.3</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:3">
       <c r="A38" s="3">
         <v>46320</v>
       </c>
@@ -2329,7 +2300,7 @@
         <v>71.61</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:3">
       <c r="A39" s="3">
         <v>46320</v>
       </c>
@@ -2340,7 +2311,7 @@
         <v>77.3</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:3">
       <c r="A40" s="3">
         <v>46320</v>
       </c>
@@ -2348,10 +2319,10 @@
         <v>15</v>
       </c>
       <c r="C40">
-        <v>82.99</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+        <v>82.98999999999999</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
       <c r="A41" s="3">
         <v>46320</v>
       </c>
@@ -2362,7 +2333,7 @@
         <v>88.3</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:3">
       <c r="A42" s="3">
         <v>46320</v>
       </c>
@@ -2373,7 +2344,7 @@
         <v>92.86</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:3">
       <c r="A43" s="3">
         <v>46320</v>
       </c>
@@ -2381,10 +2352,10 @@
         <v>18</v>
       </c>
       <c r="C43">
-        <v>96.35</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+        <v>96.34999999999999</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3">
       <c r="A44" s="3">
         <v>46320</v>
       </c>
@@ -2395,7 +2366,7 @@
         <v>98.55</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:3">
       <c r="A45" s="3">
         <v>46320</v>
       </c>
@@ -2406,7 +2377,7 @@
         <v>99.3</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:3">
       <c r="A46" s="3">
         <v>46320</v>
       </c>
@@ -2417,7 +2388,7 @@
         <v>98.55</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:3">
       <c r="A47" s="3">
         <v>46320</v>
       </c>
@@ -2425,10 +2396,10 @@
         <v>22</v>
       </c>
       <c r="C47">
-        <v>96.35</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+        <v>96.34999999999999</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3">
       <c r="A48" s="3">
         <v>46320</v>
       </c>
@@ -2439,7 +2410,7 @@
         <v>92.86</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:3">
       <c r="A49" s="3">
         <v>46320</v>
       </c>
@@ -2450,7 +2421,7 @@
         <v>88.3</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:3">
       <c r="A50" s="3">
         <v>46320</v>
       </c>
@@ -2458,10 +2429,10 @@
         <v>25</v>
       </c>
       <c r="C50">
-        <v>82.99</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+        <v>82.98999999999999</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3">
       <c r="A51" s="3">
         <v>46321</v>
       </c>
@@ -2469,10 +2440,10 @@
         <v>1</v>
       </c>
       <c r="C51">
-        <v>82.29</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+        <v>82.29000000000001</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3">
       <c r="A52" s="3">
         <v>46321</v>
       </c>
@@ -2480,10 +2451,10 @@
         <v>2</v>
       </c>
       <c r="C52">
-        <v>76.599999999999994</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+        <v>76.59999999999999</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3">
       <c r="A53" s="3">
         <v>46321</v>
       </c>
@@ -2494,7 +2465,7 @@
         <v>70.91</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:3">
       <c r="A54" s="3">
         <v>46321</v>
       </c>
@@ -2502,10 +2473,10 @@
         <v>4</v>
       </c>
       <c r="C54">
-        <v>65.599999999999994</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
+        <v>65.59999999999999</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3">
       <c r="A55" s="3">
         <v>46321</v>
       </c>
@@ -2516,7 +2487,7 @@
         <v>61.04</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:3">
       <c r="A56" s="3">
         <v>46321</v>
       </c>
@@ -2527,7 +2498,7 @@
         <v>57.55</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:3">
       <c r="A57" s="3">
         <v>46321</v>
       </c>
@@ -2538,7 +2509,7 @@
         <v>55.35</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:3">
       <c r="A58" s="3">
         <v>46321</v>
       </c>
@@ -2549,7 +2520,7 @@
         <v>54.6</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:3">
       <c r="A59" s="3">
         <v>46321</v>
       </c>
@@ -2560,7 +2531,7 @@
         <v>55.35</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:3">
       <c r="A60" s="3">
         <v>46321</v>
       </c>
@@ -2571,7 +2542,7 @@
         <v>57.55</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:3">
       <c r="A61" s="3">
         <v>46321</v>
       </c>
@@ -2582,7 +2553,7 @@
         <v>61.04</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:3">
       <c r="A62" s="3">
         <v>46321</v>
       </c>
@@ -2590,10 +2561,10 @@
         <v>12</v>
       </c>
       <c r="C62">
-        <v>65.599999999999994</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+        <v>65.59999999999999</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3">
       <c r="A63" s="3">
         <v>46321</v>
       </c>
@@ -2601,10 +2572,10 @@
         <v>14</v>
       </c>
       <c r="C63">
-        <v>76.599999999999994</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+        <v>76.59999999999999</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3">
       <c r="A64" s="3">
         <v>46321</v>
       </c>
@@ -2612,10 +2583,10 @@
         <v>15</v>
       </c>
       <c r="C64">
-        <v>82.29</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+        <v>82.29000000000001</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3">
       <c r="A65" s="3">
         <v>46321</v>
       </c>
@@ -2623,10 +2594,10 @@
         <v>16</v>
       </c>
       <c r="C65">
-        <v>87.6</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+        <v>87.59999999999999</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3">
       <c r="A66" s="3">
         <v>46321</v>
       </c>
@@ -2637,7 +2608,7 @@
         <v>92.16</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:3">
       <c r="A67" s="3">
         <v>46321</v>
       </c>
@@ -2645,10 +2616,10 @@
         <v>18</v>
       </c>
       <c r="C67">
-        <v>95.65</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
+        <v>95.65000000000001</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3">
       <c r="A68" s="3">
         <v>46321</v>
       </c>
@@ -2656,10 +2627,10 @@
         <v>19</v>
       </c>
       <c r="C68">
-        <v>97.85</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
+        <v>97.84999999999999</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3">
       <c r="A69" s="3">
         <v>46321</v>
       </c>
@@ -2667,10 +2638,10 @@
         <v>20</v>
       </c>
       <c r="C69">
-        <v>98.6</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+        <v>98.59999999999999</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3">
       <c r="A70" s="3">
         <v>46321</v>
       </c>
@@ -2678,10 +2649,10 @@
         <v>21</v>
       </c>
       <c r="C70">
-        <v>97.85</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
+        <v>97.84999999999999</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3">
       <c r="A71" s="3">
         <v>46321</v>
       </c>
@@ -2689,10 +2660,10 @@
         <v>22</v>
       </c>
       <c r="C71">
-        <v>95.65</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
+        <v>95.65000000000001</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3">
       <c r="A72" s="3">
         <v>46321</v>
       </c>
@@ -2703,7 +2674,7 @@
         <v>92.16</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:3">
       <c r="A73" s="3">
         <v>46321</v>
       </c>
@@ -2711,10 +2682,10 @@
         <v>24</v>
       </c>
       <c r="C73">
-        <v>87.6</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
+        <v>87.59999999999999</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3">
       <c r="A74" s="3">
         <v>46322</v>
       </c>
@@ -2725,7 +2696,7 @@
         <v>83.69</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:3">
       <c r="A75" s="3">
         <v>46322</v>
       </c>
@@ -2736,7 +2707,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:3">
       <c r="A76" s="3">
         <v>46322</v>
       </c>
@@ -2747,7 +2718,7 @@
         <v>72.31</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:3">
       <c r="A77" s="3">
         <v>46322</v>
       </c>
@@ -2758,7 +2729,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:3">
       <c r="A78" s="3">
         <v>46322</v>
       </c>
@@ -2769,7 +2740,7 @@
         <v>62.44</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:3">
       <c r="A79" s="3">
         <v>46322</v>
       </c>
@@ -2780,7 +2751,7 @@
         <v>58.95</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:3">
       <c r="A80" s="3">
         <v>46322</v>
       </c>
@@ -2791,7 +2762,7 @@
         <v>56.75</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:3">
       <c r="A81" s="3">
         <v>46322</v>
       </c>
@@ -2802,7 +2773,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:3">
       <c r="A82" s="3">
         <v>46322</v>
       </c>
@@ -2813,7 +2784,7 @@
         <v>56.75</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:3">
       <c r="A83" s="3">
         <v>46322</v>
       </c>
@@ -2824,7 +2795,7 @@
         <v>58.95</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:3">
       <c r="A84" s="3">
         <v>46322</v>
       </c>
@@ -2835,7 +2806,7 @@
         <v>62.44</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:3">
       <c r="A85" s="3">
         <v>46322</v>
       </c>
@@ -2846,7 +2817,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:3">
       <c r="A86" s="3">
         <v>46322</v>
       </c>
@@ -2857,7 +2828,7 @@
         <v>72.31</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:3">
       <c r="A87" s="3">
         <v>46322</v>
       </c>
@@ -2868,7 +2839,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:3">
       <c r="A88" s="3">
         <v>46322</v>
       </c>
@@ -2879,7 +2850,7 @@
         <v>83.69</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:3">
       <c r="A89" s="3">
         <v>46322</v>
       </c>
@@ -2890,7 +2861,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:3">
       <c r="A90" s="3">
         <v>46322</v>
       </c>
@@ -2901,7 +2872,7 @@
         <v>93.56</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:3">
       <c r="A91" s="3">
         <v>46322</v>
       </c>
@@ -2912,7 +2883,7 @@
         <v>97.05</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:3">
       <c r="A92" s="3">
         <v>46322</v>
       </c>
@@ -2923,7 +2894,7 @@
         <v>99.25</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:3">
       <c r="A93" s="3">
         <v>46322</v>
       </c>
@@ -2934,7 +2905,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:3">
       <c r="A94" s="3">
         <v>46322</v>
       </c>
@@ -2945,7 +2916,7 @@
         <v>99.25</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:3">
       <c r="A95" s="3">
         <v>46322</v>
       </c>
@@ -2956,7 +2927,7 @@
         <v>97.05</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:3">
       <c r="A96" s="3">
         <v>46322</v>
       </c>
@@ -2967,7 +2938,7 @@
         <v>93.56</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:3">
       <c r="A97" s="3">
         <v>46322</v>
       </c>
@@ -2984,14 +2955,14 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="6" width="16.6640625" customWidth="1"/>
+    <col min="1" max="6" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>

</xml_diff>